<commit_message>
BatchTest & WebSkill & TransportManual
</commit_message>
<xml_diff>
--- a/test/Sample_BatchTest.xlsx
+++ b/test/Sample_BatchTest.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\takas\Downloads\analytics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B81C5A00-1942-46D3-8647-85DAACCA944D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38351204-E1B1-4F65-AAA8-8F93B296F02E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="42420" yWindow="3890" windowWidth="18720" windowHeight="12420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1140" yWindow="1140" windowWidth="18720" windowHeight="11650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test" sheetId="1" r:id="rId1"/>
@@ -25,14 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
-  <si>
-    <t>設問</t>
-    <rPh sb="0" eb="2">
-      <t>セツモン</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>あなたは誰ですか？</t>
     <rPh sb="4" eb="5">
@@ -119,10 +112,19 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>回答例</t>
-    <rPh sb="0" eb="3">
-      <t>カイトウレイ</t>
-    </rPh>
+    <t>Question</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Ground Truth</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Compare</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Answer</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -473,60 +475,66 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="40.58203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="29.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="8.6640625" style="1"/>
+    <col min="2" max="4" width="29.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:4">
       <c r="A1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>11</v>
+      <c r="C2" s="1" t="s">
+        <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
+    <row r="3" spans="1:4">
+      <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="C5" s="1" t="s">
+        <v>3</v>
+      </c>
     </row>
-    <row r="3" spans="1:2">
-      <c r="A3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="1" t="s">
+    <row r="6" spans="1:4">
+      <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>